<commit_message>
Report and workbook v1.1
Report restyled to the 1STAND palette with recoloured maps and the research
URL on the cover. Workbook gains a published-at block listing every file and
the live pages.
</commit_message>
<xml_diff>
--- a/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
+++ b/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1175,6 +1175,102 @@
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>were unaffected: both years parsed identically, so matching never depended on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>PUBLISHED AT</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Findings</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>1stand.org/research/tarrant-county-closed-149-polling-places</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Interactive map</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>munsdev.github.io/1stand-embeds/tarrant-polling/standalone.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Printable report</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>munsdev.github.io/1stand-embeds/tarrant-polling/tarrant_polling_closures_report.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>This workbook</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>munsdev.github.io/1stand-embeds/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Closures CSV</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>munsdev.github.io/1stand-embeds/tarrant-polling/tarrant_closed_sites_2022_to_2026.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Coordinates</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>munsdev.github.io/1stand-embeds/tarrant-polling/tarrant_coords.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr"/>
+      <c r="B83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>v1.1, 3 September 2026. Addresses corrected and coordinates added since v1.0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Distinguish the adopted plan from the tabled August proposal
Adds the competing-count note, the 76104 clarification and tighter sourcing
on figures that come from the coalition letter rather than from this analysis.
</commit_message>
<xml_diff>
--- a/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
+++ b/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1271,6 +1271,134 @@
       <c r="B84" s="2" t="inlineStr">
         <is>
           <t>v1.1, 3 September 2026. Addresses corrected and coordinates added since v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>WHICH PLAN THESE FIGURES DESCRIBE</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Adopted plan</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>This workbook describes the Election Day list adopted 1 September 2026 and published</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr"/>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2 September: 223 rows against 316 in 2022. Commissioners approved 224; the published list</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr"/>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>has 223 and had not been amended as of 4 September.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Tabled plan</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>A proposal tabled 4 August 2026 would have left 176 Election Day sites and 42 early voting</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr"/>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>sites. Counts of 186 closed and 46 opened, which appear in some trackers, describe that</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr"/>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>tabled proposal, not this one. 316 - 186 + 46 = 176.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr"/>
+      <c r="B93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>ZIP 76104</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Some coverage names 76104 as the ZIP left with no site. That originates in public testimony</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr"/>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>on 1 September about the pre-vote proposal and was repeated in syndicated copy. On the</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr"/>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>adopted list 76104 has three sites, down from seven. 76103 is the only ZIP that reaches zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr"/>
+      <c r="B97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Not our figures</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Wait-time counts and the 'no site under 20 voters' figure come from the NAACP LDF coalition</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr"/>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>letter of 28 August 2026, sourced there to county data obtained by records request. The</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr"/>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>underlying data has not been independently reviewed here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point every link at the durable article slug
</commit_message>
<xml_diff>
--- a/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
+++ b/tarrant-polling/tarrant_polling_sites_2022_vs_2026.xlsx
@@ -942,6 +942,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
@@ -1178,6 +1179,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
@@ -1194,7 +1196,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>1stand.org/research/tarrant-county-closed-149-polling-places</t>
+          <t>1stand.org/research/tarrant-county-polling-places</t>
         </is>
       </c>
     </row>
@@ -1274,6 +1276,7 @@
         </is>
       </c>
     </row>
+    <row r="85"/>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>

</xml_diff>